<commit_message>
Atualização automática - 25/05/2026 11:13
</commit_message>
<xml_diff>
--- a/Aplicativos/GAM/bd_entrada/ajustepp.xlsx
+++ b/Aplicativos/GAM/bd_entrada/ajustepp.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="18">
   <si>
     <t>CODIGO_PRODUTO</t>
   </si>
@@ -50,9 +50,6 @@
     <t>MAXIMO</t>
   </si>
   <si>
-    <t>TEMP CAMPERO LINGUICA CASEIRA 60G C PIMENTA</t>
-  </si>
-  <si>
     <t>DIAS_RELATORIO_VENDA</t>
   </si>
   <si>
@@ -74,25 +71,19 @@
     <t>Status</t>
   </si>
   <si>
-    <t>CR DEN SORRISO 70G TRIPLA LIMPEZA COMPLETA</t>
-  </si>
-  <si>
-    <t>ACHOC PO NESCAU LT 350G</t>
-  </si>
-  <si>
-    <t>DET LIQ ATRIUS 5L GLICA</t>
-  </si>
-  <si>
-    <t>ENERG RED BULL MACA S A LT 250ML</t>
-  </si>
-  <si>
-    <t>DET PO OMO LAVAGEM PERFEITA 700G</t>
-  </si>
-  <si>
-    <t>KIT CASA CLEAN BANHEIRO 910ML</t>
-  </si>
-  <si>
-    <t>KIT CASA CLEAN COZINHA 910ML</t>
+    <t>SUCO SKINKA 450 ML UVA</t>
+  </si>
+  <si>
+    <t>VERMUTE MARTINI 750ML TINTO</t>
+  </si>
+  <si>
+    <t>BARR STO ANTONIO AMENDOBAR WHEY 40G ORIG</t>
+  </si>
+  <si>
+    <t>PAPEL HIG SULINO NEUTRO FS 30M C 4</t>
+  </si>
+  <si>
+    <t>PE MOLEQUE STO ANTONIO AC MASC MEL 200G</t>
   </si>
 </sst>
 </file>
@@ -432,7 +423,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M58"/>
+  <dimension ref="A1:M35"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="49.42578125" bestFit="1" customWidth="1"/>
@@ -458,482 +449,482 @@
         <v>5</v>
       </c>
       <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="L1" t="s">
-        <v>12</v>
-      </c>
       <c r="M1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:13">
       <c r="A2">
-        <v>3755</v>
+        <v>8532</v>
       </c>
       <c r="B2" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="C2">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="E2">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="F2">
-        <v>27</v>
+        <v>53</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3">
-        <v>3755</v>
+        <v>8732</v>
       </c>
       <c r="B3" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="C3">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="D3">
         <v>2</v>
       </c>
       <c r="E3">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="F3">
-        <v>27</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4">
-        <v>3755</v>
+        <v>8732</v>
       </c>
       <c r="B4" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="C4">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="D4">
         <v>3</v>
       </c>
       <c r="E4">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F4">
-        <v>27</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5">
-        <v>3755</v>
+        <v>8732</v>
       </c>
       <c r="B5" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="C5">
+        <v>12</v>
+      </c>
+      <c r="D5">
+        <v>6</v>
+      </c>
+      <c r="E5">
+        <v>6</v>
+      </c>
+      <c r="F5">
         <v>18</v>
-      </c>
-      <c r="D5">
-        <v>4</v>
-      </c>
-      <c r="E5">
-        <v>9</v>
-      </c>
-      <c r="F5">
-        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6">
-        <v>3755</v>
+        <v>8732</v>
       </c>
       <c r="B6" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="C6">
+        <v>12</v>
+      </c>
+      <c r="D6">
+        <v>11</v>
+      </c>
+      <c r="E6">
+        <v>6</v>
+      </c>
+      <c r="F6">
         <v>18</v>
-      </c>
-      <c r="D6">
-        <v>5</v>
-      </c>
-      <c r="E6">
-        <v>9</v>
-      </c>
-      <c r="F6">
-        <v>27</v>
       </c>
     </row>
     <row r="7" spans="1:13">
       <c r="A7">
-        <v>5244</v>
+        <v>8732</v>
       </c>
       <c r="B7" t="s">
         <v>14</v>
       </c>
       <c r="C7">
-        <v>144</v>
+        <v>12</v>
       </c>
       <c r="D7">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="E7">
-        <v>144</v>
+        <v>6</v>
       </c>
       <c r="F7">
-        <v>288</v>
+        <v>18</v>
       </c>
     </row>
     <row r="8" spans="1:13">
       <c r="A8">
-        <v>5244</v>
+        <v>8732</v>
       </c>
       <c r="B8" t="s">
         <v>14</v>
       </c>
       <c r="C8">
-        <v>144</v>
+        <v>12</v>
       </c>
       <c r="D8">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="E8">
-        <v>144</v>
+        <v>6</v>
       </c>
       <c r="F8">
-        <v>288</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9" spans="1:13">
       <c r="A9">
-        <v>5244</v>
+        <v>8732</v>
       </c>
       <c r="B9" t="s">
         <v>14</v>
       </c>
       <c r="C9">
-        <v>144</v>
+        <v>12</v>
       </c>
       <c r="D9">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="E9">
-        <v>144</v>
+        <v>6</v>
       </c>
       <c r="F9">
-        <v>288</v>
+        <v>18</v>
       </c>
     </row>
     <row r="10" spans="1:13">
       <c r="A10">
-        <v>5244</v>
+        <v>8732</v>
       </c>
       <c r="B10" t="s">
         <v>14</v>
       </c>
       <c r="C10">
-        <v>144</v>
+        <v>12</v>
       </c>
       <c r="D10">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="E10">
-        <v>144</v>
+        <v>6</v>
       </c>
       <c r="F10">
-        <v>288</v>
+        <v>18</v>
       </c>
     </row>
     <row r="11" spans="1:13">
       <c r="A11">
-        <v>5244</v>
+        <v>8732</v>
       </c>
       <c r="B11" t="s">
         <v>14</v>
       </c>
       <c r="C11">
-        <v>144</v>
+        <v>12</v>
       </c>
       <c r="D11">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="E11">
-        <v>144</v>
+        <v>6</v>
       </c>
       <c r="F11">
-        <v>288</v>
+        <v>18</v>
       </c>
     </row>
     <row r="12" spans="1:13">
       <c r="A12">
-        <v>5244</v>
+        <v>13072</v>
       </c>
       <c r="B12" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C12">
         <v>144</v>
       </c>
       <c r="D12">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E12">
-        <v>144</v>
+        <v>44</v>
       </c>
       <c r="F12">
-        <v>288</v>
+        <v>188</v>
       </c>
     </row>
     <row r="13" spans="1:13">
       <c r="A13">
-        <v>5244</v>
+        <v>13072</v>
       </c>
       <c r="B13" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C13">
         <v>144</v>
       </c>
       <c r="D13">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E13">
-        <v>144</v>
+        <v>44</v>
       </c>
       <c r="F13">
-        <v>288</v>
+        <v>188</v>
       </c>
     </row>
     <row r="14" spans="1:13">
       <c r="A14">
-        <v>5244</v>
+        <v>13072</v>
       </c>
       <c r="B14" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C14">
         <v>144</v>
       </c>
       <c r="D14">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="E14">
-        <v>144</v>
+        <v>44</v>
       </c>
       <c r="F14">
-        <v>288</v>
+        <v>188</v>
       </c>
     </row>
     <row r="15" spans="1:13">
       <c r="A15">
-        <v>5244</v>
+        <v>13072</v>
       </c>
       <c r="B15" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C15">
         <v>144</v>
       </c>
       <c r="D15">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="E15">
-        <v>144</v>
+        <v>44</v>
       </c>
       <c r="F15">
-        <v>288</v>
+        <v>188</v>
       </c>
     </row>
     <row r="16" spans="1:13">
       <c r="A16">
-        <v>5244</v>
+        <v>13072</v>
       </c>
       <c r="B16" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C16">
         <v>144</v>
       </c>
       <c r="D16">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="E16">
-        <v>144</v>
+        <v>44</v>
       </c>
       <c r="F16">
-        <v>288</v>
+        <v>188</v>
       </c>
     </row>
     <row r="17" spans="1:6">
       <c r="A17">
-        <v>5244</v>
+        <v>13072</v>
       </c>
       <c r="B17" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C17">
         <v>144</v>
       </c>
       <c r="D17">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="E17">
-        <v>144</v>
+        <v>44</v>
       </c>
       <c r="F17">
-        <v>288</v>
+        <v>188</v>
       </c>
     </row>
     <row r="18" spans="1:6">
       <c r="A18">
-        <v>5244</v>
+        <v>21700</v>
       </c>
       <c r="B18" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C18">
-        <v>144</v>
+        <v>20</v>
       </c>
       <c r="D18">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="E18">
-        <v>144</v>
+        <v>12</v>
       </c>
       <c r="F18">
-        <v>288</v>
+        <v>32</v>
       </c>
     </row>
     <row r="19" spans="1:6">
       <c r="A19">
-        <v>12216</v>
+        <v>21700</v>
       </c>
       <c r="B19" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C19">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="D19">
         <v>2</v>
       </c>
       <c r="E19">
-        <v>244</v>
+        <v>16</v>
       </c>
       <c r="F19">
-        <v>316</v>
+        <v>36</v>
       </c>
     </row>
     <row r="20" spans="1:6">
       <c r="A20">
-        <v>12216</v>
+        <v>21700</v>
       </c>
       <c r="B20" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C20">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="D20">
         <v>3</v>
       </c>
       <c r="E20">
-        <v>360</v>
+        <v>40</v>
       </c>
       <c r="F20">
-        <v>432</v>
+        <v>60</v>
       </c>
     </row>
     <row r="21" spans="1:6">
       <c r="A21">
-        <v>12216</v>
+        <v>21700</v>
       </c>
       <c r="B21" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C21">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="D21">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E21">
-        <v>244</v>
+        <v>20</v>
       </c>
       <c r="F21">
-        <v>316</v>
+        <v>40</v>
       </c>
     </row>
     <row r="22" spans="1:6">
       <c r="A22">
-        <v>17336</v>
+        <v>21700</v>
       </c>
       <c r="B22" t="s">
         <v>16</v>
       </c>
       <c r="C22">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="D22">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E22">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="F22">
-        <v>70</v>
+        <v>40</v>
       </c>
     </row>
     <row r="23" spans="1:6">
       <c r="A23">
-        <v>37250</v>
+        <v>21700</v>
       </c>
       <c r="B23" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C23">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D23">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E23">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="F23">
-        <v>40</v>
+        <v>50</v>
       </c>
     </row>
     <row r="24" spans="1:6">
       <c r="A24">
-        <v>37250</v>
+        <v>21700</v>
       </c>
       <c r="B24" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C24">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D24">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E24">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="F24">
         <v>40</v>
@@ -941,73 +932,73 @@
     </row>
     <row r="25" spans="1:6">
       <c r="A25">
-        <v>37250</v>
+        <v>21700</v>
       </c>
       <c r="B25" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C25">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D25">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E25">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="F25">
-        <v>40</v>
+        <v>30</v>
       </c>
     </row>
     <row r="26" spans="1:6">
       <c r="A26">
-        <v>37250</v>
+        <v>21700</v>
       </c>
       <c r="B26" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C26">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D26">
         <v>11</v>
       </c>
       <c r="E26">
-        <v>12</v>
+        <v>40</v>
       </c>
       <c r="F26">
-        <v>36</v>
+        <v>60</v>
       </c>
     </row>
     <row r="27" spans="1:6">
       <c r="A27">
-        <v>37250</v>
+        <v>21700</v>
       </c>
       <c r="B27" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C27">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D27">
         <v>12</v>
       </c>
       <c r="E27">
-        <v>12</v>
+        <v>40</v>
       </c>
       <c r="F27">
-        <v>36</v>
+        <v>60</v>
       </c>
     </row>
     <row r="28" spans="1:6">
       <c r="A28">
-        <v>37250</v>
+        <v>21700</v>
       </c>
       <c r="B28" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C28">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D28">
         <v>13</v>
@@ -1016,24 +1007,24 @@
         <v>12</v>
       </c>
       <c r="F28">
-        <v>36</v>
+        <v>32</v>
       </c>
     </row>
     <row r="29" spans="1:6">
       <c r="A29">
-        <v>37250</v>
+        <v>21700</v>
       </c>
       <c r="B29" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C29">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D29">
         <v>14</v>
       </c>
       <c r="E29">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F29">
         <v>36</v>
@@ -1041,582 +1032,122 @@
     </row>
     <row r="30" spans="1:6">
       <c r="A30">
-        <v>37250</v>
+        <v>21700</v>
       </c>
       <c r="B30" t="s">
+        <v>16</v>
+      </c>
+      <c r="C30">
+        <v>20</v>
+      </c>
+      <c r="D30">
         <v>17</v>
       </c>
-      <c r="C30">
-        <v>24</v>
-      </c>
-      <c r="D30">
-        <v>18</v>
-      </c>
       <c r="E30">
-        <v>12</v>
+        <v>40</v>
       </c>
       <c r="F30">
-        <v>36</v>
+        <v>60</v>
       </c>
     </row>
     <row r="31" spans="1:6">
       <c r="A31">
-        <v>37776</v>
+        <v>21700</v>
       </c>
       <c r="B31" t="s">
+        <v>16</v>
+      </c>
+      <c r="C31">
+        <v>20</v>
+      </c>
+      <c r="D31">
         <v>18</v>
       </c>
-      <c r="C31">
-        <v>20</v>
-      </c>
-      <c r="D31">
-        <v>1</v>
-      </c>
       <c r="E31">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="F31">
-        <v>32</v>
+        <v>40</v>
       </c>
     </row>
     <row r="32" spans="1:6">
       <c r="A32">
-        <v>37776</v>
+        <v>21784</v>
       </c>
       <c r="B32" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C32">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="D32">
         <v>2</v>
       </c>
       <c r="E32">
-        <v>36</v>
+        <v>6</v>
       </c>
       <c r="F32">
-        <v>56</v>
+        <v>16</v>
       </c>
     </row>
     <row r="33" spans="1:6">
       <c r="A33">
-        <v>37776</v>
+        <v>21784</v>
       </c>
       <c r="B33" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C33">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="D33">
         <v>3</v>
       </c>
       <c r="E33">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="F33">
-        <v>68</v>
+        <v>16</v>
       </c>
     </row>
     <row r="34" spans="1:6">
       <c r="A34">
-        <v>37776</v>
+        <v>21784</v>
       </c>
       <c r="B34" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C34">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="D34">
         <v>4</v>
       </c>
       <c r="E34">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F34">
-        <v>32</v>
+        <v>16</v>
       </c>
     </row>
     <row r="35" spans="1:6">
       <c r="A35">
-        <v>37776</v>
+        <v>21784</v>
       </c>
       <c r="B35" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C35">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="D35">
         <v>5</v>
       </c>
       <c r="E35">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F35">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6">
-      <c r="A36">
-        <v>37776</v>
-      </c>
-      <c r="B36" t="s">
-        <v>18</v>
-      </c>
-      <c r="C36">
-        <v>20</v>
-      </c>
-      <c r="D36">
-        <v>6</v>
-      </c>
-      <c r="E36">
-        <v>36</v>
-      </c>
-      <c r="F36">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6">
-      <c r="A37">
-        <v>37776</v>
-      </c>
-      <c r="B37" t="s">
-        <v>18</v>
-      </c>
-      <c r="C37">
-        <v>20</v>
-      </c>
-      <c r="D37">
-        <v>7</v>
-      </c>
-      <c r="E37">
-        <v>24</v>
-      </c>
-      <c r="F37">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6">
-      <c r="A38">
-        <v>37776</v>
-      </c>
-      <c r="B38" t="s">
-        <v>18</v>
-      </c>
-      <c r="C38">
-        <v>20</v>
-      </c>
-      <c r="D38">
-        <v>8</v>
-      </c>
-      <c r="E38">
-        <v>24</v>
-      </c>
-      <c r="F38">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6">
-      <c r="A39">
-        <v>37776</v>
-      </c>
-      <c r="B39" t="s">
-        <v>18</v>
-      </c>
-      <c r="C39">
-        <v>20</v>
-      </c>
-      <c r="D39">
-        <v>11</v>
-      </c>
-      <c r="E39">
-        <v>36</v>
-      </c>
-      <c r="F39">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6">
-      <c r="A40">
-        <v>37776</v>
-      </c>
-      <c r="B40" t="s">
-        <v>18</v>
-      </c>
-      <c r="C40">
-        <v>20</v>
-      </c>
-      <c r="D40">
-        <v>12</v>
-      </c>
-      <c r="E40">
-        <v>36</v>
-      </c>
-      <c r="F40">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6">
-      <c r="A41">
-        <v>37776</v>
-      </c>
-      <c r="B41" t="s">
-        <v>18</v>
-      </c>
-      <c r="C41">
-        <v>20</v>
-      </c>
-      <c r="D41">
-        <v>13</v>
-      </c>
-      <c r="E41">
-        <v>24</v>
-      </c>
-      <c r="F41">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6">
-      <c r="A42">
-        <v>37776</v>
-      </c>
-      <c r="B42" t="s">
-        <v>18</v>
-      </c>
-      <c r="C42">
-        <v>20</v>
-      </c>
-      <c r="D42">
-        <v>14</v>
-      </c>
-      <c r="E42">
-        <v>24</v>
-      </c>
-      <c r="F42">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6">
-      <c r="A43">
-        <v>37776</v>
-      </c>
-      <c r="B43" t="s">
-        <v>18</v>
-      </c>
-      <c r="C43">
-        <v>20</v>
-      </c>
-      <c r="D43">
-        <v>17</v>
-      </c>
-      <c r="E43">
-        <v>36</v>
-      </c>
-      <c r="F43">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6">
-      <c r="A44">
-        <v>37776</v>
-      </c>
-      <c r="B44" t="s">
-        <v>18</v>
-      </c>
-      <c r="C44">
-        <v>20</v>
-      </c>
-      <c r="D44">
-        <v>18</v>
-      </c>
-      <c r="E44">
-        <v>48</v>
-      </c>
-      <c r="F44">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6">
-      <c r="A45">
-        <v>37840</v>
-      </c>
-      <c r="B45" t="s">
-        <v>19</v>
-      </c>
-      <c r="C45">
-        <v>5</v>
-      </c>
-      <c r="D45">
-        <v>3</v>
-      </c>
-      <c r="E45">
-        <v>20</v>
-      </c>
-      <c r="F45">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6">
-      <c r="A46">
-        <v>37840</v>
-      </c>
-      <c r="B46" t="s">
-        <v>19</v>
-      </c>
-      <c r="C46">
-        <v>5</v>
-      </c>
-      <c r="D46">
-        <v>5</v>
-      </c>
-      <c r="E46">
-        <v>10</v>
-      </c>
-      <c r="F46">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6">
-      <c r="A47">
-        <v>37840</v>
-      </c>
-      <c r="B47" t="s">
-        <v>19</v>
-      </c>
-      <c r="C47">
-        <v>5</v>
-      </c>
-      <c r="D47">
-        <v>6</v>
-      </c>
-      <c r="E47">
-        <v>15</v>
-      </c>
-      <c r="F47">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6">
-      <c r="A48">
-        <v>37840</v>
-      </c>
-      <c r="B48" t="s">
-        <v>19</v>
-      </c>
-      <c r="C48">
-        <v>5</v>
-      </c>
-      <c r="D48">
-        <v>7</v>
-      </c>
-      <c r="E48">
-        <v>10</v>
-      </c>
-      <c r="F48">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6">
-      <c r="A49">
-        <v>37840</v>
-      </c>
-      <c r="B49" t="s">
-        <v>19</v>
-      </c>
-      <c r="C49">
-        <v>5</v>
-      </c>
-      <c r="D49">
-        <v>8</v>
-      </c>
-      <c r="E49">
-        <v>10</v>
-      </c>
-      <c r="F49">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6">
-      <c r="A50">
-        <v>37840</v>
-      </c>
-      <c r="B50" t="s">
-        <v>19</v>
-      </c>
-      <c r="C50">
-        <v>5</v>
-      </c>
-      <c r="D50">
-        <v>11</v>
-      </c>
-      <c r="E50">
-        <v>20</v>
-      </c>
-      <c r="F50">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6">
-      <c r="A51">
-        <v>37840</v>
-      </c>
-      <c r="B51" t="s">
-        <v>19</v>
-      </c>
-      <c r="C51">
-        <v>5</v>
-      </c>
-      <c r="D51">
-        <v>12</v>
-      </c>
-      <c r="E51">
-        <v>20</v>
-      </c>
-      <c r="F51">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="52" spans="1:6">
-      <c r="A52">
-        <v>37840</v>
-      </c>
-      <c r="B52" t="s">
-        <v>19</v>
-      </c>
-      <c r="C52">
-        <v>5</v>
-      </c>
-      <c r="D52">
-        <v>13</v>
-      </c>
-      <c r="E52">
-        <v>10</v>
-      </c>
-      <c r="F52">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="53" spans="1:6">
-      <c r="A53">
-        <v>37840</v>
-      </c>
-      <c r="B53" t="s">
-        <v>19</v>
-      </c>
-      <c r="C53">
-        <v>5</v>
-      </c>
-      <c r="D53">
-        <v>14</v>
-      </c>
-      <c r="E53">
-        <v>10</v>
-      </c>
-      <c r="F53">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="54" spans="1:6">
-      <c r="A54">
-        <v>37840</v>
-      </c>
-      <c r="B54" t="s">
-        <v>19</v>
-      </c>
-      <c r="C54">
-        <v>5</v>
-      </c>
-      <c r="D54">
-        <v>17</v>
-      </c>
-      <c r="E54">
-        <v>15</v>
-      </c>
-      <c r="F54">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="55" spans="1:6">
-      <c r="A55">
-        <v>37840</v>
-      </c>
-      <c r="B55" t="s">
-        <v>19</v>
-      </c>
-      <c r="C55">
-        <v>5</v>
-      </c>
-      <c r="D55">
-        <v>18</v>
-      </c>
-      <c r="E55">
-        <v>15</v>
-      </c>
-      <c r="F55">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="56" spans="1:6">
-      <c r="A56">
-        <v>37841</v>
-      </c>
-      <c r="B56" t="s">
-        <v>20</v>
-      </c>
-      <c r="C56">
-        <v>5</v>
-      </c>
-      <c r="D56">
-        <v>11</v>
-      </c>
-      <c r="E56">
-        <v>15</v>
-      </c>
-      <c r="F56">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="57" spans="1:6">
-      <c r="A57">
-        <v>37841</v>
-      </c>
-      <c r="B57" t="s">
-        <v>20</v>
-      </c>
-      <c r="C57">
-        <v>5</v>
-      </c>
-      <c r="D57">
-        <v>17</v>
-      </c>
-      <c r="E57">
-        <v>15</v>
-      </c>
-      <c r="F57">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="58" spans="1:6">
-      <c r="A58">
-        <v>37841</v>
-      </c>
-      <c r="B58" t="s">
-        <v>20</v>
-      </c>
-      <c r="C58">
-        <v>5</v>
-      </c>
-      <c r="D58">
-        <v>18</v>
-      </c>
-      <c r="E58">
-        <v>15</v>
-      </c>
-      <c r="F58">
-        <v>20</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>